<commit_message>
Update debates data - 2026-06-12
</commit_message>
<xml_diff>
--- a/Debats_SEM_Migration.xlsx
+++ b/Debats_SEM_Migration.xlsx
@@ -62,15 +62,14 @@
     <t xml:space="preserve">DE</t>
   </si>
   <si>
-    <t xml:space="preserve">Ihre Aussenpolitische Kommission stimmte am 23. März dem Abkommen zwischen dem Schweizerischen Bundesrat und dem Ministerkabinett der Ukraine über die Zusammenarbeit im Wiederaufbauprozess der Ukraine mit 19 zu 0 Stimmen bei 6 Enthaltungen zu. 
-Beim Wiederaufbau der Ukraine ist insbesondere im Energie- und Infrastrukturbereich ein verstärktes Engagement privater Unternehmen notwendig, sinnvoll und erwünscht. Das vorliegende bilaterale Abkommen schafft die rechtliche Grundlage dafür. Die Ukraine </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ihre Aussenpolitische Kommission stimmte am 23. März dem Abkommen zwischen dem Schweizerischen Bundesrat und dem Ministerkabinett der Ukraine über die Zusammenarbeit im Wiederaufbauprozess der Ukraine mit 19 zu 0 Stimmen bei 6 Enthaltungen zu. 
-Beim Wiederaufbau der Ukraine ist insbesondere im Energie- und Infrastrukturbereich ein verstärktes Engagement privater Unternehmen notwendig, sinnvoll und erwünscht. Das vorliegende bilaterale Abkommen schafft die rechtliche Grundlage dafür. Die Ukraine kann Güter und Dienstleistungen definieren, welche die Schweiz anschliessend im Rahmen des bewilligten Budgets bei Schweizer Unternehmen gemäss öffentlichem Beschaffungsrecht, aber unter Ausschluss ausländischer Anbieter, beschafft. Mit dem Abkommen werden Expertise und Innovation aus der Schweiz stärker genutzt und private Investitionen mobilisiert. Auf diese Weise leistet die Schweiz einen Beitrag zum Wiederaufbau der ukrainischen Infrastruktur und Wirtschaft. Die Einbindung der Schweizer Privatwirtschaft in den Wiederaufbau ist einer der Schwerpunkte des Länderprogramms Ukraine 2025-2028 der IZA.
-Im Rahmen der Beratung wurden zwei Anträge auf eine Kommissionsmotion abgehandelt. Die erste Kommissionsmotion zielt auf die Zuweisung von vorgesehenen Mitteln an ein UN-Wiederaufbauinstrument anstelle einer Verknüpfung mit der Schweizer Privatindustrie. Die Kommission lehnte diesen Antrag mit 16 zu 6 Stimmen bei 3 Enthaltungen ab. Ein weiterer Antrag auf eine Kommissionsmotion zur Verknüpfung des Abkommens mit der Auflösung des Schutzstatus S für ukrainische Staatsangehörige aus stabilen Herkunftsregionen wurde mit 16 zu 9 Stimmen ebenfalls abgelehnt. 
-Schliesslich wurde ein Antrag auf einen neuen Artikel 1 Absatz 3, im Bundesbeschluss bezüglich der Rücksichtnahme auf die Empfehlungen des Development Assistance Committee (DAC) der OECD mit 13 zu 12 Stimmen angenommen. Das DAC erlässt unter anderem Umsetzungsrichtlinien für die Entwicklungszusammenarbeit.
-Die Minderheit Rüegger will diesen neuen Absatz 3 zur Verknüpfung mit den OECD-Richtlinien streichen. Sie findet, dass die DAC-Regeln für Entwicklungshilfe zu eng gefasst sind und den Spielraum für Schweizer Unternehmen bei der Unterstützung des Wiederaufbaus unnötigerweise einengen.
+    <t xml:space="preserve">Ihre Aussenpolitische Kommission stimmte am 23.[NB]März dem Abkommen zwischen dem Schweizerischen Bundesrat und dem Ministerkabinett der Ukraine über die Zusammenarbeit im Wiederaufbauprozess der Ukraine mit 19 zu 0 Stimmen bei 6 Enthaltungen zu. 
+Beim Wiederaufbau der Ukraine ist insbesondere im Energie- und Infrastrukturbereich ein verstärktes Engagement privater Unternehmen notwendig, sinnvoll und erwünscht. Das vorliegende bilaterale Abkommen schafft die rechtliche Grundlage dafür. Die Ukrai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ihre Aussenpolitische Kommission stimmte am 23.[NB]März dem Abkommen zwischen dem Schweizerischen Bundesrat und dem Ministerkabinett der Ukraine über die Zusammenarbeit im Wiederaufbauprozess der Ukraine mit 19 zu 0 Stimmen bei 6 Enthaltungen zu. 
+Beim Wiederaufbau der Ukraine ist insbesondere im Energie- und Infrastrukturbereich ein verstärktes Engagement privater Unternehmen notwendig, sinnvoll und erwünscht. Das vorliegende bilaterale Abkommen schafft die rechtliche Grundlage dafür. Die Ukraine kann Güter und Dienstleistungen definieren, welche die Schweiz anschliessend im Rahmen des bewilligten Budgets bei Schweizer Unternehmen gemäss öffentlichem Beschaffungsrecht, aber unter Ausschluss ausländischer Anbieter beschafft. Mit dem Abkommen werden Expertise und Innovation aus der Schweiz stärker genutzt und private Investitionen mobilisiert. Auf diese Weise leistet die Schweiz einen Beitrag zum Wiederaufbau der ukrainischen Infrastruktur und Wirtschaft. Die Einbindung der Schweizer Privatwirtschaft in den Wiederaufbau ist einer der Schwerpunkte des Länderprogramms Ukraine 2025-2028 der IZA.
+Im Rahmen der Beratung wurden zwei Anträge auf eine Kommissionsmotion abgehandelt. Der erste Antrag auf eine Kommissionsmotion zielte auf die Zuweisung von vorgesehenen Mitteln an ein UN-Wiederaufbauinstrument anstelle einer Verknüpfung mit der Schweizer Privatindustrie. Die Kommission lehnte diesen Antrag mit 16 zu 6 Stimmen bei 3 Enthaltungen ab. Ein weiterer Antrag auf eine Kommissionsmotion zur Verknüpfung des Abkommens mit der Auflösung des Schutzstatus S für ukrainische Staatsangehörige aus stabilen Herkunftsregionen wurde mit 16 zu 9 Stimmen ebenfalls abgelehnt. 
+Schliesslich wurde ein Antrag auf einen neuen Artikel 1 Absatz 3 im Bundesbeschluss bezüglich der Rücksichtnahme auf die Empfehlungen des Development Assistance Committee (DAC) der OECD mit 13 zu 12 Stimmen angenommen. Das DAC erlässt unter anderem Umsetzungsrichtlinien für die Entwicklungszusammenarbeit. Die Minderheit Rüegger will diesen neuen Absatz 3 zur Verknüpfung mit den OECD-Richtlinien streichen. Sie findet, dass die DAC-Regeln für Entwicklungshilfe zu eng gefasst sind und den Spielraum für Schweizer Unternehmen bei der Unterstützung des Wiederaufbaus unnötigerweise einengen.
 </t>
   </si>
   <si>
@@ -92,7 +91,7 @@
 Schon meine Vorrednerin der Grünen Fraktion hat gesagt - auch uns ist das wichtig -, dass im Abkommen einige andere Themen geregelt werden, so zum Beispiel das Thema der Korruption. Wir müssen hier nicht einfach so tun, als ob wir es mit einem total unbescholtenen Partnerstaat zu tun hätten, mit dem wir ein solches Abkommen machen. Die Ukraine hat in vielen Dingen, wie etwa bei den Menschenrechten, bei der Korruption und bei anderen Sachen, noch nicht den Standard, den wir uns wünschen. Trotzdem glauben wir, dass wir mit diesem Beitrag zum Wiederaufbau der Ukraine auch helfen können. Zudem ist auch die Streitschlichtung, die in diesem Abkommen ebenfalls behandelt wird, gerecht und auf Augenhöhe geregelt.
 Was ich aber nicht verstehe, ist, dass der Antrag für Artikel 1 Absatz 3 eine Mehrheit bekommen hat. Hier schaue ich zur Mitte-Fraktion: Dieser Antrag hat eine Mehrheit bekommen, weil Ihre Mitglieder in der APK - es ist kein Kommissionsgeheimnis, Sie können es hier selber herausfinden - ihm zugestimmt haben. Auch Sie sangen erst das Hohelied auf die privatwirtschaftliche Wiederaufbauhilfe, und nun torpedieren Sie diese genau mit diesem Absatz. Die Minderheitssprecherin, Kollegin Rüegger, hat die Details eigentlich exzellent erklärt.
 Lassen Sie mich noch etwas Weiteres sagen: Es handelt sich hier um eine Arbeitsgruppe innerhalb der OECD. Jetzt müssen Sie sich vorstellen, dass diese Arbeitsgruppe, in der rund dreissig andere Länder vertreten sind, dieses Abkommen durchgeht, dieses analysiert und uns dann sagt, was sie findet, was wir tun dürfen und was wir nicht tun dürfen. Diese Arbeitsgruppe wird eben genau auch einen ihrer Grundsätze einbringen, wonach man nämlich die eigene Wirtschaft zum Beispiel nicht mit Entwicklungshilfe begünstigen darf. Aber genau das wollten wir, das ist in der IZA-Strategie so festgehalten, das haben wir auch im Budget so festgehalten. Ich möchte die Mitte-Fraktion daher doch bitten, wieder von diesem Absatz wegzukommen und den Antrag der Minderheit Rüegger zu unterstützen. 
-Lassen Sie mich noch ein Schlusswort sagen. Weshalb leisten wir Wiederaufbauhilfe für die Ukraine? Es ist eine Schwerpunktregion für uns, sie ist in unserer Nachbarschaft, und wir haben alles Interesse daran - sei es beim Thema Migration, sei es beim Thema Sicherheit oder aber auch bei wirtschaftlichen Themen -, dass wir mit der Ukraine eine gute Partnerschaft haben und dass die Ukraine wieder auf die Beine kommt. Aber es ist kein Schuldbekenntnis von uns. Als ich vor dem Pfingstwochenende am Treffen des EWR-Parlamentarierkomitees war, sagte ich, was die Schweiz macht. Ich sagte aber auch: Die Schweiz ist weder Kriegspartei, noch ist es unser Krieg. Und mir hat tatsächlich die Aussenministerin von Liechtenstein im Namen der EWR-Minister widersprochen und gesagt: Doch, das ist unser Krieg, und wir sind Kriegspartei, und deshalb müssen wir der Ukraine beistehen. Nein - und das ist meine persönliche Meinung -: Wir stehen der Ukraine bei, weil sie ungerechtfertigt von einem Aggressor angegriffen wurde, weil sie zerstört wird, weil dort menschliches Leid geschieht. Aber wir stehen der Ukraine nicht bei, weil dies unser Krieg ist oder weil wir Kriegspartei sind.
+Lassen Sie mich noch ein Schlusswort sagen. Weshalb leisten wir Wiederaufbauhilfe für die Ukraine? Es ist eine Schwerpunktregion für uns, sie ist in unserer Nachbarschaft, und wir haben alles Interesse daran - sei es beim Thema Migration, sei es beim Thema Sicherheit oder aber auch bei wirtschaftlichen Themen -, dass wir mit der Ukraine eine gute Partnerschaft haben und dass die Ukraine wieder auf die Beine kommt. Aber es ist kein Schuldbekenntnis von uns. Als ich vor dem Pfingstwochenende am Treffen des EWR-Parlamentarierkomitees war, sagte ich, was die Schweiz macht. Ich sagte aber auch: Die Schweiz ist weder Kriegspartei, noch ist es unser Krieg. Und mir hat tatsächlich die Aussenministerin von Liechtenstein im Namen der EWR-Minister widersprochen und gesagt: "Doch, das ist unser Krieg, und wir sind Kriegspartei, und deshalb müssen wir der Ukraine beistehen." Nein, und das ist meine persönliche Meinung, wir stehen der Ukraine bei, weil sie ungerechtfertigt von einem Aggressor angegriffen wurde, weil sie zerstört wird, weil dort menschliches Leid geschieht. Aber wir stehen der Ukraine nicht bei, weil dies unser Krieg ist oder weil wir Kriegspartei sind.
 </t>
   </si>
   <si>
@@ -666,17 +665,17 @@
     <t xml:space="preserve">Barandun Nicole</t>
   </si>
   <si>
-    <t xml:space="preserve">Seit 1999, wir haben es schon gehört, beteiligt sich die Schweizer Armee mit Swisscoy an der KFOR, der Nato-geführten, aber von der UNO mandatierten Friedensmission in Kosovo. 
+    <t xml:space="preserve">Seit 1999, wir haben es schon gehört, beteiligt sich die Schweizer Armee mit Swisscoy an der Kfor, der Nato-geführten, aber von der UNO mandatierten Friedensmission in Kosovo. 
 Die Sicherheitslage im Kosovo ist aktuell ruhig, sie bleibt aber weiterhin volatil. Sie ist, ausdrücklich gesagt, nicht stabil, so schätzen es auch unsere europäischen Nachbarländer ein. Insbesondere im Norden sind die Spannungen anhaltend hoch. Erst 2023 kam es zu schweren Sicherheitsvorfällen, die die Nato gleich zweima</t>
   </si>
   <si>
-    <t xml:space="preserve">Seit 1999, wir haben es schon gehört, beteiligt sich die Schweizer Armee mit Swisscoy an der KFOR, der Nato-geführten, aber von der UNO mandatierten Friedensmission in Kosovo. 
-Die Sicherheitslage im Kosovo ist aktuell ruhig, sie bleibt aber weiterhin volatil. Sie ist, ausdrücklich gesagt, nicht stabil, so schätzen es auch unsere europäischen Nachbarländer ein. Insbesondere im Norden sind die Spannungen anhaltend hoch. Erst 2023 kam es zu schweren Sicherheitsvorfällen, die die Nato gleich zweimal zur Verstärkung der KFOR zwangen. Solange die Beziehungen zwischen Kosovo und Serbien nicht nachhaltig normalisiert sind, halten die Nato und die beteiligten Staaten die KFOR für notwendig, als militärische Garantin eines sicheren Umfelds, die Entwicklung und Stabilität im Kosovo und auf dem gesamten Westbalkan gewährleistet.
+    <t xml:space="preserve">Seit 1999, wir haben es schon gehört, beteiligt sich die Schweizer Armee mit Swisscoy an der Kfor, der Nato-geführten, aber von der UNO mandatierten Friedensmission in Kosovo. 
+Die Sicherheitslage im Kosovo ist aktuell ruhig, sie bleibt aber weiterhin volatil. Sie ist, ausdrücklich gesagt, nicht stabil, so schätzen es auch unsere europäischen Nachbarländer ein. Insbesondere im Norden sind die Spannungen anhaltend hoch. Erst 2023 kam es zu schweren Sicherheitsvorfällen, die die Nato gleich zweimal zur Verstärkung der Kfor zwangen. Solange die Beziehungen zwischen Kosovo und Serbien nicht nachhaltig normalisiert sind, halten die Nato und die beteiligten Staaten die Kfor für notwendig, als militärische Garantin eines sicheren Umfelds, die Entwicklung und Stabilität im Kosovo und auf dem gesamten Westbalkan gewährleistet.
 Die Schweiz leistet mit Swisscoy seit 25 Jahren einen verlässlichen Beitrag zu dieser Stabilität, und sie leistet diesen Beitrag auch mit ganz konkreten Handlungen. Ich spreche zum Beispiel die Liaison and Monitoring Teams an, die im direkten Austausch mit der Bevölkerung Spannungen früh erkennen und versuchen, diese zu entschärfen, aber auch unsere Genietruppen, die vor Ort wichtige Dienste leisten u. a. in der Logistik. Darüber hinaus kann die Schweizer Armee mit dem Einsatz wichtige Erfahrungen in einer internationalen Operation sammeln, die auch für unsere Verteidigungsfähigkeit hier zuhause relevant sind. 
 Die Schweiz hat ein direktes Interesse am Frieden, an der Stabilität und an der wirtschaftlichen Entwicklung des Kosovos und der ganzen Region. Der Westbalkan ist für uns sicherheits-, migrations- und wirtschaftspolitisch relevant. Wir haben aufgrund der engen menschlichen und wirtschaftlichen Beziehungen auch Verpflichtungen gegenüber dieser Region. Mit der Verlängerung unseres Engagements übernehmen wir Verantwortung. Diese Verantwortung tragen wir, weil wir eine enge Beziehung zu dieser Region pflegen. 
 Ich möchte noch ein Wort zur kosovarischen Diaspora in der Schweiz verlieren. Infolge des Kosovokriegs fanden Ende der Neunzigerjahre rund 60 000 Menschen aus dem Kosovo vorübergehend Schutz in der Schweiz. Viele von ihnen sind später zurückgekehrt, aber ein Teil von ihnen hat hier dauerhaft Fuss gefasst. Ihre Kinder und Enkelkinder sind heute ein selbstverständlicher Teil unserer Gesellschaft. Insgesamt leben in der Schweiz deutlich über 100 000 Menschen mit Wurzeln im Kosovo; Schätzungen sprechen von rund 170 000 Kosovo-Albanerinnen und -Albanern. Aus migrationspolitischer Sicht wissen wir, wenn es wieder zu einer schweren Eskalation käme, würden sich die neuen Fluchtbewegungen dorthin richten, wo bereits Familien und etablierte Netzwerke bestehen. Für die Schweiz mit ihrer grossen kosovarischen Community sind Prävention und Stabilität im Kosovo daher auch migrationspolitisch sinnvoll. Das Risiko eines erneuten unkontrollierten Flüchtlingsstroms wird dadurch reduziert anstatt erhöht. 
-Ich sage noch ein Wort zur Neutralität. Sie schwebt immer ein bisschen mit im Raum. Das Mandat der KFOR basiert auf einem klaren Mandat des UNO-Sicherheitsrates. Es handelt sich um eine klassische friedensfördernde Operation. Die Neutralität steht solchen von der UNO mandatierten Friedensoperationen gerade nicht entgegen. Die Schweizer Beteiligung entspricht einer seit Jahren gefestigten Praxis der schweizerischen Aussen- und Sicherheitspolitik. 
-Ich empfehle Ihnen im Namen der Mitte-Fraktion. Die Mitte. EVP, dieser Vorlage zuzustimmen, das heisst, einzutreten und der Mehrheit zu folgen. Bei der Erhöhung des Kontingents geht es um einen Maximalrahmen, nicht um einen Automatismus. Der Bundesrat bleibt dem Parlament gegenüber verantwortlich. Verteidigungsfähigkeit entsteht nicht in einem Vakuum. Wer eine glaubwürdige Landesverteidigung will, braucht gut ausgebildete Kader mit realer Einsatzerfahrung. Die KFOR bleibt vor dem Hintergrund einer nach wie vor volatilen Lage im Kosovo und einer ungelösten Beziehung zu Serbien deshalb auch aus Sicht der Schweiz notwendig. 
+Ich sage noch ein Wort zur Neutralität. Sie schwebt immer ein bisschen mit im Raum. Das Mandat der Kfor basiert auf einem klaren Mandat des UNO-Sicherheitsrates. Es handelt sich um eine klassische friedensfördernde Operation. Die Neutralität steht solchen von der UNO mandatierten Friedensoperationen gerade nicht entgegen. Die Schweizer Beteiligung entspricht einer seit Jahren gefestigten Praxis der schweizerischen Aussen- und Sicherheitspolitik. 
+Ich empfehle Ihnen im Namen der Mitte-Fraktion. Die Mitte. EVP, dieser Vorlage zuzustimmen, das heisst, einzutreten und der Mehrheit zu folgen. Bei der Erhöhung des Kontingents geht es um einen Maximalrahmen, nicht um einen Automatismus. Der Bundesrat bleibt dem Parlament gegenüber verantwortlich. Verteidigungsfähigkeit entsteht nicht in einem Vakuum. Wer eine glaubwürdige Landesverteidigung will, braucht gut ausgebildete Kader mit realer Einsatzerfahrung. Die Kfor bleibt vor dem Hintergrund einer nach wie vor volatilen Lage im Kosovo und einer ungelösten Beziehung zu Serbien deshalb auch aus Sicht der Schweiz notwendig. 
 </t>
   </si>
   <si>

</xml_diff>